<commit_message>
adding 4.2026.9 Release frameworks
</commit_message>
<xml_diff>
--- a/March_Release_SCB/Cypress/fixtures/AgencyTemplate.xlsx
+++ b/March_Release_SCB/Cypress/fixtures/AgencyTemplate.xlsx
@@ -466,10 +466,10 @@
         <v/>
       </c>
       <c r="C2" t="str">
-        <v>757375</v>
+        <v>574487</v>
       </c>
       <c r="D2" t="str">
-        <v>Natalie</v>
+        <v>Chase</v>
       </c>
       <c r="E2" t="str">
         <v>2256</v>
@@ -499,10 +499,10 @@
         <v>wiki field</v>
       </c>
       <c r="N2" t="str">
-        <v>4722119024</v>
+        <v>4639857937</v>
       </c>
       <c r="O2" t="str">
-        <v>natalie@yopmail.com</v>
+        <v>chase@yopmail.com</v>
       </c>
       <c r="P2" t="str">
         <v>12-10-2022</v>

</xml_diff>